<commit_message>
Add NKON pricing and refresh battery candidates
</commit_message>
<xml_diff>
--- a/dist/Mooch_21700_2026-09-21.xlsx
+++ b/dist/Mooch_21700_2026-09-21.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Фото 11.08.2026" sheetId="1" r:id="Rfd26524e024c46e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Форум" sheetId="2" r:id="R906b833397104b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Методика" sheetId="3" r:id="R1c645950bd564ed4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Фото 11.08.2026" sheetId="1" r:id="R97f39dc99ec94f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Форум" sheetId="2" r:id="R57685ebb51ff4519"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Методика" sheetId="3" r:id="Rba842b8be10b4b1a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ForumTests" displayName="ForumTests" ref="A1:N51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ForumTests" displayName="ForumTests" ref="A1:N52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Модель / версия"/>
     <x:tableColumn id="2" name="Ёмкость в заголовке, мА·ч"/>
@@ -2725,7 +2725,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24717e5de2fe40e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2e7c375f714584"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4530,10 +4530,50 @@
         <x:v>2026-09-21</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A52" s="6" t="str">
+        <x:v>Samsung 50S</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C52" s="9" t="n">
+        <x:v>44784</x:v>
+      </x:c>
+      <x:c r="D52" s="7" t="n">
+        <x:v>5049</x:v>
+      </x:c>
+      <x:c r="E52" s="7" t="n">
+        <x:v>5071</x:v>
+      </x:c>
+      <x:c r="F52" s="8"/>
+      <x:c r="G52" s="8"/>
+      <x:c r="H52" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I52" s="8" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J52" s="6" t="str">
+        <x:v>Текст статьи прочитан</x:v>
+      </x:c>
+      <x:c r="K52" s="6" t="str">
+        <x:v>Паспортная версия 50S рассчитана на 25 А continuous и 45 А только до 80 °C. В повторном тесте оба образца превысили 85 °C при 25 А до 2,5 В, поэтому Mooch рекомендует не более 20 А непрерывно. Не объединять с Samsung 50S2.</x:v>
+      </x:c>
+      <x:c r="L52" s="6" t="str">
+        <x:v>https://www.e-cigarette-forum.com/threads/bench-test-results-samsung-50s-25a-5000mah-21700.975569/</x:v>
+      </x:c>
+      <x:c r="M52" s="6" t="str">
+        <x:v>Bench Test Results: Samsung 50S - 25A 5000mAh 21700</x:v>
+      </x:c>
+      <x:c r="N52" s="1" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0f13f8c56314859"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44f0dd653e234572"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4559,7 +4599,7 @@
         <x:v>Охват</x:v>
       </x:c>
       <x:c r="B2" s="10" t="str">
-        <x:v>41 строка фото с ёмкостью строго более 4000 мА·ч и 50 тем форума. Полный текст структурирован у 47 статей; три записи остались ссылками без извлечения текста.</x:v>
+        <x:v>41 строка фото с ёмкостью строго более 4000 мА·ч и 51 тем форума. Полный текст структурирован у 48 статей; три записи остались ссылками без извлечения текста.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
@@ -4631,7 +4671,7 @@
         <x:v>Доступность</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Структурированные данные извлечены из 47 статей; 3 записи содержат только заголовок и ссылку. Парсинг не подтверждает наличие товара в продаже.</x:v>
+        <x:v>Структурированные данные извлечены из 48 статей; 3 записи содержат только заголовок и ссылку. Парсинг не подтверждает наличие товара в продаже.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">

</xml_diff>

<commit_message>
Publish battery study revision 10
</commit_message>
<xml_diff>
--- a/dist/Mooch_21700_2026-09-21.xlsx
+++ b/dist/Mooch_21700_2026-09-21.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Фото 11.08.2026" sheetId="1" r:id="R97f39dc99ec94f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Форум" sheetId="2" r:id="R57685ebb51ff4519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Методика" sheetId="3" r:id="Rba842b8be10b4b1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Фото 11.08.2026" sheetId="1" r:id="Rdc518e6aa25b4d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Форум" sheetId="2" r:id="R6df6f141e0904989"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Методика" sheetId="3" r:id="R67e6316c099a40e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2725,7 +2725,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2e7c375f714584"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dcbf3d070854a5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4496,7 +4496,7 @@
         <x:v>2026-09-21</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="51" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A51" s="6" t="str">
         <x:v>Samsung 50S2</x:v>
       </x:c>
@@ -4506,20 +4506,30 @@
       <x:c r="C51" s="9" t="n">
         <x:v>45695</x:v>
       </x:c>
-      <x:c r="D51" s="7"/>
-      <x:c r="E51" s="7"/>
+      <x:c r="D51" s="7" t="n">
+        <x:v>5111</x:v>
+      </x:c>
+      <x:c r="E51" s="7" t="n">
+        <x:v>5143</x:v>
+      </x:c>
       <x:c r="F51" s="8" t="n">
         <x:v>12.9</x:v>
       </x:c>
       <x:c r="G51" s="8" t="n">
         <x:v>13.8</x:v>
       </x:c>
-      <x:c r="H51" s="8"/>
-      <x:c r="I51" s="8"/>
+      <x:c r="H51" s="8" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I51" s="8" t="n">
+        <x:v>45</x:v>
+      </x:c>
       <x:c r="J51" s="6" t="str">
         <x:v>Текст статьи прочитан</x:v>
       </x:c>
-      <x:c r="K51" s="6"/>
+      <x:c r="K51" s="6" t="str">
+        <x:v>Обновлённая версия 50S. При 5 и 25 А работала немного дольше и на 4–7 °C холоднее исходной 50S; разница времени заметна главным образом ниже 3,0–3,1 В. 45 А допускаются только до 80 °C. Mooch отметил различия между партиями и необходимость входного контроля. Не объединять с Samsung 50S.</x:v>
+      </x:c>
       <x:c r="L51" s="6" t="str">
         <x:v>https://www.e-cigarette-forum.com/threads/bench-test-results-samsung-50s2-25a-45a-5000mah-21700.988832/</x:v>
       </x:c>
@@ -4530,7 +4540,7 @@
         <x:v>2026-09-21</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="52" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A52" s="6" t="str">
         <x:v>Samsung 50S</x:v>
       </x:c>
@@ -4558,7 +4568,7 @@
         <x:v>Текст статьи прочитан</x:v>
       </x:c>
       <x:c r="K52" s="6" t="str">
-        <x:v>Паспортная версия 50S рассчитана на 25 А continuous и 45 А только до 80 °C. В повторном тесте оба образца превысили 85 °C при 25 А до 2,5 В, поэтому Mooch рекомендует не более 20 А непрерывно. Не объединять с Samsung 50S2.</x:v>
+        <x:v>Паспортная версия 50S рассчитана на 25 А continuous и 45 А только до 80 °C. В повторном тесте оба образца превысили 85 °C при 25 А до 2,5 В, поэтому Mooch рекомендует не более 20 А непрерывно. Отдельный источник 18650pro оценивает сопротивление примерно в 10 мОм. На графике до 2,8 В максимумы температуры составили 41/51/63/73/85/95 °C при 5/10/15/20/25/30 А. Не объединять с Samsung 50S2.</x:v>
       </x:c>
       <x:c r="L52" s="6" t="str">
         <x:v>https://www.e-cigarette-forum.com/threads/bench-test-results-samsung-50s-25a-5000mah-21700.975569/</x:v>
@@ -4573,7 +4583,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44f0dd653e234572"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8182b3882ead46de"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>